<commit_message>
feat(documents): per-vendor branded PDF/Excel/Word (logos, brand colours, template variants); seed passes category-accurate brand; 302/302 parse-back intact
</commit_message>
<xml_diff>
--- a/public/seed/atlascloud-iaas/atlascloud-iaas-invoice-2025-07.xlsx
+++ b/public/seed/atlascloud-iaas/atlascloud-iaas-invoice-2025-07.xlsx
@@ -5,17 +5,21 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Document" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Remittance" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="67">
   <si>
     <t>Invoice AC-INV-01 — AtlasCloud (IaaS)</t>
   </si>
   <si>
+    <t>AtlasCloud (IaaS)</t>
+  </si>
+  <si>
     <t>__docType</t>
   </si>
   <si>
@@ -25,9 +29,6 @@
     <t>__vendorName</t>
   </si>
   <si>
-    <t>AtlasCloud (IaaS)</t>
-  </si>
-  <si>
     <t>Field</t>
   </si>
   <si>
@@ -206,13 +207,19 @@
   </si>
   <si>
     <t>$3,000.00</t>
+  </si>
+  <si>
+    <t>AT</t>
+  </si>
+  <si>
+    <t>Remit to AtlasCloud (IaaS) — please reference the document title on all payments.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -222,21 +229,64 @@
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0E7490"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="FF9CA3AF"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0E7490"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1F2937"/>
+    </font>
+    <font>
+      <color rgb="FF1F2937"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0E7490"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
-      <b/>
+      <i/>
+      <color rgb="FF1F2937"/>
+      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0E7490"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EEF2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -244,15 +294,62 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF0E7490"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF0E7490"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF0E7490"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -592,292 +689,346 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" defaultColWidth="24"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>3</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B8" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="B9" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B10" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B11" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B12" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B13" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B14" s="6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B15" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="B16" s="6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B17" s="8" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B18" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B19" s="8" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B20" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B21" s="8" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B22" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="9" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+    <row r="25" ht="18" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B25" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C25" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D25" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="E25" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F25" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="G23" s="3" t="s">
+      <c r="G25" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="H23" s="3" t="s">
+      <c r="H25" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="I23" s="3" t="s">
+      <c r="I25" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="J23" s="3" t="s">
+      <c r="J25" s="10" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B26" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C26" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D26" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E26" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="F26" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="G26" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="H24" s="2" t="s">
+      <c r="H26" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="I24" s="2" t="s">
+      <c r="I26" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="J24" s="2" t="s">
+      <c r="J26" s="6" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B27" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C27" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="D27" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E27" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="F27" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G25" s="2" t="s">
+      <c r="G27" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="H25" s="2" t="s">
+      <c r="H27" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="I27" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="J25" s="2" t="s">
+      <c r="J27" s="8" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B28" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C28" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D28" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E28" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F28" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="G26" s="2" t="s">
+      <c r="G28" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="H26" s="2" t="s">
+      <c r="H28" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="I26" s="2" t="s">
+      <c r="I28" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="J26" s="2" t="s">
+      <c r="J28" s="6" t="s">
         <v>52</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" defaultColWidth="24"/>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:G3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>